<commit_message>
Version 1.0.0.99, Se actualizan GPID, Pañol
</commit_message>
<xml_diff>
--- a/Recursos/Tablas/GPID.xlsx
+++ b/Recursos/Tablas/GPID.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/56746e89e6462cb5/01-Onedrive-matiaschamu/02-Trabajos/02-Programacion (Varios)/03-Proyectos_Android/02-SolTec/SolTecPep/Tablas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matia\Documents\GitHub Repos\Soltec\Recursos\Tablas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{D78F35F9-C1ED-4781-9938-147D268CF59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5824CB3-5435-468F-BC68-219EA8B4EDC0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F654931-944D-4A75-B39A-AA90D658FBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Arcidiacono Pablo </t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Leo Jorge</t>
+  </si>
+  <si>
+    <t>Lucas Rojas</t>
   </si>
 </sst>
 </file>
@@ -149,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -184,91 +187,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -277,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -291,31 +219,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -598,14 +514,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="25.53515625" customWidth="1"/>
+    <col min="2" max="2" width="12.69140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="16.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>16</v>
       </c>
@@ -613,7 +529,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -621,7 +537,7 @@
         <v>30159771</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
@@ -629,15 +545,15 @@
         <v>80000711</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="5">
         <v>30162827</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -645,15 +561,15 @@
         <v>30159772</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="5">
         <v>30159774</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -661,15 +577,15 @@
         <v>40250752</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+    <row r="8" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="5">
         <v>40250751</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -677,15 +593,15 @@
         <v>30162874</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="9">
         <v>40251370</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
@@ -693,15 +609,15 @@
         <v>80102645</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="9">
         <v>80060729</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
@@ -709,15 +625,15 @@
         <v>80034291</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="9">
         <v>80139460</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
         <v>13</v>
       </c>
@@ -725,15 +641,15 @@
         <v>80200118</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="9">
         <v>80218156</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="6" t="s">
         <v>15</v>
       </c>
@@ -741,12 +657,20 @@
         <v>40251711</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:2" ht="15.9" x14ac:dyDescent="0.4">
+      <c r="A18" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="13">
+      <c r="B18" s="9">
         <v>40251261</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="7">
+        <v>81289321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>